<commit_message>
feat: Implement configurable duplicate prefix for transaction detection
</commit_message>
<xml_diff>
--- a/temp/BBVA_ACCOUNT_20250210.xlsx
+++ b/temp/BBVA_ACCOUNT_20250210.xlsx
@@ -471,8 +471,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>-28820</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>-28820,0</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -496,8 +498,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>-13479.26</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>-13479,26</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -521,8 +525,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>-1010605.89</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-1010605,89</t>
+        </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -546,8 +552,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>-388095</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-388095,0</t>
+        </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -571,8 +579,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>1441000</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1441000,0</t>
+        </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -596,8 +606,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>0.15</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0,15</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -621,8 +633,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>194.9</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>194,9</t>
+        </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -646,8 +660,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>-194.9</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>-194,9</t>
+        </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -671,8 +687,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>-9745.43</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>-9745,43</t>
+        </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -696,8 +714,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>50000</v>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>50000,0</t>
+        </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -721,8 +741,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>9745.43</v>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>9745,43</t>
+        </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -746,8 +768,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>-29990</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>-29990,0</t>
+        </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -771,8 +795,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>-19990</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>-19990,0</t>
+        </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -796,8 +822,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>-10</v>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>-10,0</t>
+        </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -821,8 +849,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>-10</v>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>-10,0</t>
+        </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -846,8 +876,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>-90072.88</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>-90072,88</t>
+        </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -871,8 +903,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>90072.88</v>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>90072,88</t>
+        </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -896,8 +930,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>-39574.32</v>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>-39574,32</t>
+        </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -921,8 +957,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>-185170</v>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>-185170,0</t>
+        </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -946,8 +984,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>-3480</v>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>-3480,0</t>
+        </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -971,8 +1011,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>-1095461.57</v>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>-1095461,57</t>
+        </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -996,8 +1038,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>1323685.52</v>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>1323685,52</t>
+        </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1021,8 +1065,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>-0.01</v>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>-0,01</t>
+        </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1046,8 +1092,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>-10000</v>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>-10000,0</t>
+        </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1071,8 +1119,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>0.38</v>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>0,38</t>
+        </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1096,8 +1146,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D27" t="n">
-        <v>10000</v>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>10000,0</t>
+        </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1121,8 +1173,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>-89952.53</v>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>-89952,53</t>
+        </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1146,8 +1200,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>89952.53</v>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>89952,53</t>
+        </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1171,8 +1227,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>-61724.82</v>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>-61724,82</t>
+        </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1196,8 +1254,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>-1549449.84</v>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>-1549449,84</t>
+        </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1221,8 +1281,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D32" t="n">
-        <v>-508042.7</v>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>-508042,7</t>
+        </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1246,8 +1308,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>2119217.32</v>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2119217,32</t>
+        </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1271,8 +1335,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>0.04</v>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>0,04</t>
+        </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1296,8 +1362,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>-1200</v>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>-1200,0</t>
+        </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1321,8 +1389,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>1200</v>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>1200,0</t>
+        </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1346,8 +1416,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D37" t="n">
-        <v>-100000</v>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>-100000,0</t>
+        </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1371,8 +1443,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D38" t="n">
-        <v>-100000</v>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>-100000,0</t>
+        </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1396,8 +1470,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D39" t="n">
-        <v>-100000</v>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>-100000,0</t>
+        </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1421,8 +1497,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D40" t="n">
-        <v>-100000</v>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>-100000,0</t>
+        </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1446,8 +1524,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D41" t="n">
-        <v>400000</v>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>400000,0</t>
+        </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1471,8 +1551,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D42" t="n">
-        <v>-129564</v>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>-129564,0</t>
+        </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1496,8 +1578,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>129564</v>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>129564,0</t>
+        </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1521,8 +1605,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D44" t="n">
-        <v>-29644.23</v>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>-29644,23</t>
+        </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1546,8 +1632,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D45" t="n">
-        <v>-120000.21</v>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>-120000,21</t>
+        </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1571,8 +1659,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D46" t="n">
-        <v>-91380</v>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>-91380,0</t>
+        </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1596,8 +1686,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D47" t="n">
-        <v>-49846.4</v>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>-49846,4</t>
+        </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1621,8 +1713,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D48" t="n">
-        <v>-938294.62</v>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>-938294,62</t>
+        </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1646,8 +1740,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D49" t="n">
-        <v>120000</v>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>120000,0</t>
+        </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1671,8 +1767,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D50" t="n">
-        <v>91380</v>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>91380,0</t>
+        </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1696,8 +1794,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D51" t="n">
-        <v>1017785.25</v>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>1017785,25</t>
+        </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1721,8 +1821,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D52" t="n">
-        <v>0.21</v>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>0,21</t>
+        </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1746,8 +1848,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D53" t="n">
-        <v>-2860</v>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>-2860,0</t>
+        </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1771,8 +1875,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D54" t="n">
-        <v>2860</v>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2860,0</t>
+        </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1796,8 +1902,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D55" t="n">
-        <v>-80000</v>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>-80000,0</t>
+        </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1821,8 +1929,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D56" t="n">
-        <v>80000</v>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>80000,0</t>
+        </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1846,8 +1956,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D57" t="n">
-        <v>-37949.67</v>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>-37949,67</t>
+        </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1871,8 +1983,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D58" t="n">
-        <v>-89010</v>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>-89010,0</t>
+        </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1896,8 +2010,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D59" t="n">
-        <v>-1166285.11</v>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>-1166285,11</t>
+        </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1921,8 +2037,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D60" t="n">
-        <v>1292953.96</v>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>1292953,96</t>
+        </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1946,8 +2064,10 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D61" t="n">
-        <v>290.82</v>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>290,82</t>
+        </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>

</xml_diff>